<commit_message>
Add laboratory labels under LA chart X-axis products
Show Laboratorio A–J below each product tick, grouping shared labs
(B for LA2–LA3, E for LA6–LA7), and include Laboratorio in the Excel data.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/la_osmolality_results.xlsx
+++ b/osmolality_results/la_osmolality_results.xlsx
@@ -241,7 +241,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$H$2:$H$13</f>
+              <f>'Data'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -269,7 +269,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$I$2:$I$13</f>
+              <f>'Data'!$J$2:$J$13</f>
             </numRef>
           </val>
         </ser>
@@ -308,12 +308,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$J$2:$J$13</f>
+              <f>'Data'!$K$2:$K$13</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$K$2:$K$13</f>
+              <f>'Data'!$L$2:$L$13</f>
             </numRef>
           </yVal>
         </ser>
@@ -346,12 +346,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$J$2:$J$13</f>
+              <f>'Data'!$K$2:$K$13</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$L$2:$L$13</f>
+              <f>'Data'!$M$2:$M$13</f>
             </numRef>
           </yVal>
         </ser>
@@ -846,21 +846,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col hidden="1" width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="14" customWidth="1" min="9" max="9"/>
-    <col hidden="1" width="10" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="12" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="14" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="10" customWidth="1" min="11" max="11"/>
     <col hidden="1" width="12" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -871,55 +872,60 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>Laboratorio</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>Spec Min (mOsm/kg)</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Spec Max (mOsm/kg)</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 (mOsm/kg)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 (mOsm/kg)</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Status</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Status</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Base (hidden)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Range Height</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>X Index</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Y</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Y</t>
         </is>
@@ -933,45 +939,50 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
+          <t>Laboratorio A</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>575</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>N/A (sin lote)</t>
         </is>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="I2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>575</v>
       </c>
-      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -979,41 +990,46 @@
           <t>LA2</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio B</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="E3" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>309</v>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>309</v>
       </c>
     </row>
@@ -1023,43 +1039,48 @@
           <t>LA3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio B</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>320</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>292</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>292</v>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
+      <c r="F4" s="4" t="n">
+        <v>292</v>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>292</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>292</v>
       </c>
+      <c r="M4" s="4" t="n">
+        <v>292</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1067,43 +1088,48 @@
           <t>LA4</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio C</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>400</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>280</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
+      <c r="F5" s="4" t="n">
+        <v>280</v>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>280</v>
       </c>
       <c r="L5" s="4" t="n">
         <v>280</v>
       </c>
+      <c r="M5" s="4" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1113,43 +1139,48 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>Laboratorio D</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>558</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>565</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>558</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>565</v>
       </c>
     </row>
@@ -1159,41 +1190,46 @@
           <t>LA6</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio E</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>304</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>304</v>
       </c>
     </row>
@@ -1203,41 +1239,46 @@
           <t>LA7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio E</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>340</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>306</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>306</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>308</v>
       </c>
     </row>
@@ -1247,41 +1288,46 @@
           <t>LA8</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio F</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>350</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>282</v>
       </c>
     </row>
@@ -1291,41 +1337,46 @@
           <t>LA9</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio G</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D10" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>292</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>292</v>
       </c>
     </row>
@@ -1335,41 +1386,46 @@
           <t>LA10</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio H</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D11" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>214</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>212</v>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>214</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>212</v>
       </c>
     </row>
@@ -1379,41 +1435,46 @@
           <t>LA11</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Laboratorio I</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>330</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>305</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>297</v>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>305</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>297</v>
       </c>
     </row>
@@ -1425,43 +1486,48 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>Laboratorio J</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>280</v>
       </c>
     </row>
@@ -1475,7 +1541,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rango de aceptación shown as a shaded band. LA1/LA5/LA12 have no specification; LA1 has Lote 1 only.</t>
+          <t>Rango de aceptación shown as a shaded band. LA1/LA5/LA12 have no specification; LA1 has Lote 1 only. X-axis shows product and belonging Laboratorio.</t>
         </is>
       </c>
     </row>
@@ -1488,8 +1554,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Tilt laboratory labels and rename LA chart X-axis
Place Laboratorio names on a slight diagonal under each product and
label the axis Laboratorio/Producto with spacing to avoid overlap.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/la_osmolality_results.xlsx
+++ b/osmolality_results/la_osmolality_results.xlsx
@@ -373,7 +373,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Producto</a:t>
+                  <a:t>Laboratorio/Producto</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1584,7 +1584,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eje X: Producto (LA1–LA12) | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2</t>
+          <t>Eje X: Producto (LA1–LA12) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Valor teórico estimado stars to LA osmolality chart
Mark LA1 and LA5 at 570 mOsm/kg and LA12 at 302 mOsm/kg using the
same star legend format as the DO chart.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/la_osmolality_results.xlsx
+++ b/osmolality_results/la_osmolality_results.xlsx
@@ -241,7 +241,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$I$2:$I$13</f>
+              <f>'Data'!$J$2:$J$13</f>
             </numRef>
           </val>
         </ser>
@@ -269,7 +269,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$J$2:$J$13</f>
+              <f>'Data'!$K$2:$K$13</f>
             </numRef>
           </val>
         </ser>
@@ -308,12 +308,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$K$2:$K$13</f>
+              <f>'Data'!$L$2:$L$13</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$L$2:$L$13</f>
+              <f>'Data'!$M$2:$M$13</f>
             </numRef>
           </yVal>
         </ser>
@@ -346,12 +346,50 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'Data'!$K$2:$K$13</f>
+              <f>'Data'!$L$2:$L$13</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Data'!$M$2:$M$13</f>
+              <f>'Data'!$N$2:$N$13</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>Valor teórico estimado</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="star"/>
+            <size val="10"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Data'!$L$2:$L$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Data'!$O$2:$O$13</f>
             </numRef>
           </yVal>
         </ser>
@@ -803,7 +841,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LA1, LA5 and LA12 have no specification range. LA1 has Lote 1 only (no Lote 2).</t>
+          <t>LA1, LA5 and LA12 have no specification range. LA1 has Lote 1 only (no Lote 2). Valor teórico estimado (*): LA1/LA5 = 570; LA12 = 302.</t>
         </is>
       </c>
     </row>
@@ -846,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -855,13 +893,15 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col hidden="1" width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="14" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="10" customWidth="1" min="11" max="11"/>
-    <col hidden="1" width="12" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="14" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="10" customWidth="1" min="12" max="12"/>
     <col hidden="1" width="12" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="12" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -897,37 +937,47 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
+          <t>Asterisk (mOsm/kg)</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
           <t>Lote 1 Status</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Status</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Base (hidden)</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Range Height</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>X Index</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Lote 1 Y</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Lote 2 Y</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Asterisk Y</t>
         </is>
       </c>
     </row>
@@ -960,29 +1010,35 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="4" t="n">
+        <v>570</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>N/A (sin lote)</t>
         </is>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>575</v>
       </c>
-      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n">
+        <v>570</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1007,31 +1063,37 @@
       <c r="F3" s="4" t="n">
         <v>309</v>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="N3" s="4" t="n">
         <v>309</v>
       </c>
+      <c r="O3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1056,31 +1118,37 @@
       <c r="F4" s="4" t="n">
         <v>292</v>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>292</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>292</v>
       </c>
+      <c r="N4" s="4" t="n">
+        <v>292</v>
+      </c>
+      <c r="O4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1105,31 +1173,37 @@
       <c r="F5" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>180</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>280</v>
       </c>
       <c r="M5" s="4" t="n">
         <v>280</v>
       </c>
+      <c r="N5" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="O5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1158,30 +1232,36 @@
       <c r="F6" s="4" t="n">
         <v>565</v>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="n">
+        <v>570</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>558</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
         <v>565</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>570</v>
       </c>
     </row>
     <row r="7">
@@ -1207,31 +1287,37 @@
       <c r="F7" s="4" t="n">
         <v>304</v>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="M7" s="4" t="n">
+      <c r="N7" s="4" t="n">
         <v>304</v>
       </c>
+      <c r="O7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1256,31 +1342,37 @@
       <c r="F8" s="4" t="n">
         <v>308</v>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>306</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>308</v>
       </c>
+      <c r="O8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1305,31 +1397,37 @@
       <c r="F9" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>281</v>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="N9" s="4" t="n">
         <v>282</v>
       </c>
+      <c r="O9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1354,31 +1452,37 @@
       <c r="F10" s="4" t="n">
         <v>292</v>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>260</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>282</v>
       </c>
-      <c r="M10" s="4" t="n">
+      <c r="N10" s="4" t="n">
         <v>292</v>
       </c>
+      <c r="O10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1403,31 +1507,37 @@
       <c r="F11" s="4" t="n">
         <v>212</v>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>160</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>214</v>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="N11" s="4" t="n">
         <v>212</v>
       </c>
+      <c r="O11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1452,31 +1562,37 @@
       <c r="F12" s="4" t="n">
         <v>297</v>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>305</v>
       </c>
-      <c r="M12" s="4" t="n">
+      <c r="N12" s="4" t="n">
         <v>297</v>
       </c>
+      <c r="O12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1505,30 +1621,36 @@
       <c r="F13" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="4" t="n">
+        <v>302</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>N/A (no specification)</t>
         </is>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="K13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>276</v>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="N13" s="4" t="n">
         <v>280</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>302</v>
       </c>
     </row>
     <row r="15">
@@ -1541,21 +1663,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Rango de aceptación shown as a shaded band. LA1/LA5/LA12 have no specification; LA1 has Lote 1 only. X-axis shows product and belonging Laboratorio.</t>
+          <t>Rango de aceptación shown as a shaded band. LA1/LA5/LA12 have no specification; LA1 has Lote 1 only. Valor teórico estimado (*): LA1/LA5 = 570; LA12 = 302.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green).</t>
+          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), estrella = Valor teórico estimado.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1584,7 +1706,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eje X: Producto (LA1–LA12) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2</t>
+          <t>Eje X: Producto (LA1–LA12) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | Estrella: Valor teórico estimado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Lágrima natural reference line at 300 mOsm/kg
Draw a navy dashed horizontal line on both DO and LA charts and include
it in the legend as Lágrima natural.

Co-authored-by: Smansilla98 <Smansilla98@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/osmolality_results/la_osmolality_results.xlsx
+++ b/osmolality_results/la_osmolality_results.xlsx
@@ -1670,7 +1670,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), estrella = Valor teórico estimado.</t>
+          <t>Units: mOsm/kg. Markers: Lote 1 (orange), Lote 2 (green), estrella = Valor teórico estimado; línea punteada azul marino = Lágrima natural (300).</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1706,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eje X: Producto (LA1–LA12) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | Estrella: Valor teórico estimado</t>
+          <t>Eje X: Producto (LA1–LA12) + Laboratorio | Eje Y: Osmolalidad (mOsm/kg), paso 25 | Sombra: Rango de aceptación | Círculos: Lote 1 &amp; Lote 2 | Estrella: Valor teórico estimado | Línea punteada: Lágrima natural (300)</t>
         </is>
       </c>
     </row>

</xml_diff>